<commit_message>
Se implementa login en portas, equipos y pre-sim. Se realizan pruebas de pre-sim
</commit_message>
<xml_diff>
--- a/src/preactivador/preactivador.xlsx
+++ b/src/preactivador/preactivador.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E106"/>
+  <dimension ref="A1:E101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,7 +458,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696905</t>
+          <t xml:space="preserve"> 57101702301638385</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -467,15 +467,21 @@
       <c r="C2" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D2" t="n">
-        <v>3135930207</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696906</t>
+          <t xml:space="preserve"> 57101702301638384</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -484,15 +490,21 @@
       <c r="C3" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D3" t="n">
-        <v>3135931096</v>
-      </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696907</t>
+          <t xml:space="preserve"> 57101702301638583</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -501,15 +513,21 @@
       <c r="C4" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D4" t="n">
-        <v>3135931941</v>
-      </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696908</t>
+          <t xml:space="preserve"> 57101702301638582</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -518,15 +536,21 @@
       <c r="C5" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D5" t="n">
-        <v>3135920112</v>
-      </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696909</t>
+          <t xml:space="preserve"> 57101702301638581</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -535,15 +559,21 @@
       <c r="C6" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D6" t="n">
-        <v>3135898951</v>
-      </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696910</t>
+          <t xml:space="preserve"> 57101702301638580</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -552,15 +582,21 @@
       <c r="C7" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D7" t="n">
-        <v>3135903811</v>
-      </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696911</t>
+          <t xml:space="preserve"> 57101702301638579</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -569,15 +605,21 @@
       <c r="C8" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D8" t="n">
-        <v>3135907550</v>
-      </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696912</t>
+          <t xml:space="preserve"> 57101702301638578</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -586,15 +628,21 @@
       <c r="C9" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D9" t="n">
-        <v>3135910106</v>
-      </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696913</t>
+          <t xml:space="preserve"> 57101702301638577</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -603,15 +651,21 @@
       <c r="C10" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D10" t="n">
-        <v>3135915186</v>
-      </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696369</t>
+          <t xml:space="preserve"> 57101702301638576</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -620,15 +674,21 @@
       <c r="C11" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D11" t="n">
-        <v>3135917708</v>
-      </c>
-      <c r="E11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696415</t>
+          <t xml:space="preserve"> 57101702301638575</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -637,15 +697,21 @@
       <c r="C12" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D12" t="n">
-        <v>3135882524</v>
-      </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696429</t>
+          <t xml:space="preserve"> 57101702301638574</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -654,15 +720,21 @@
       <c r="C13" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D13" t="n">
-        <v>3135890113</v>
-      </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696416</t>
+          <t xml:space="preserve"> 57101702301638573</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -671,15 +743,21 @@
       <c r="C14" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D14" t="n">
-        <v>3135895171</v>
-      </c>
-      <c r="E14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Validacion Causal Desactivacion IccId = Falso</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696379</t>
+          <t xml:space="preserve"> 57101702301638572</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -688,15 +766,21 @@
       <c r="C15" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D15" t="n">
-        <v>3135931512</v>
-      </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696360</t>
+          <t xml:space="preserve"> 57101702301638522</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -705,15 +789,21 @@
       <c r="C16" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D16" t="n">
-        <v>3135933512</v>
-      </c>
-      <c r="E16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696361</t>
+          <t xml:space="preserve"> 57101702301638532</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -722,15 +812,21 @@
       <c r="C17" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D17" t="n">
-        <v>3135921672</v>
-      </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696430</t>
+          <t xml:space="preserve"> 57101702301638563</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -739,15 +835,21 @@
       <c r="C18" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D18" t="n">
-        <v>3135901366</v>
-      </c>
-      <c r="E18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696364</t>
+          <t xml:space="preserve"> 57101702301638436</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -756,15 +858,21 @@
       <c r="C19" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D19" t="n">
-        <v>3135905125</v>
-      </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696376</t>
+          <t xml:space="preserve"> 57101702301638435</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -773,15 +881,21 @@
       <c r="C20" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D20" t="n">
-        <v>3135907629</v>
-      </c>
-      <c r="E20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696362</t>
+          <t xml:space="preserve"> 57101702301638434</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -790,15 +904,21 @@
       <c r="C21" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D21" t="n">
-        <v>3135912742</v>
-      </c>
-      <c r="E21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696375</t>
+          <t xml:space="preserve"> 57101702301638566</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -807,15 +927,21 @@
       <c r="C22" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D22" t="n">
-        <v>3135917782</v>
-      </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696356</t>
+          <t xml:space="preserve"> 57101702301638565</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -824,15 +950,21 @@
       <c r="C23" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D23" t="n">
-        <v>3135922531</v>
-      </c>
-      <c r="E23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696357</t>
+          <t xml:space="preserve"> 57101702301638564</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -841,15 +973,21 @@
       <c r="C24" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D24" t="n">
-        <v>3135885159</v>
-      </c>
-      <c r="E24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696358</t>
+          <t xml:space="preserve"> 57101702301638398</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -858,15 +996,21 @@
       <c r="C25" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D25" t="n">
-        <v>3135893949</v>
-      </c>
-      <c r="E25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696359</t>
+          <t xml:space="preserve"> 57101702301638397</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -875,15 +1019,21 @@
       <c r="C26" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D26" t="n">
-        <v>3135897807</v>
-      </c>
-      <c r="E26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696417</t>
+          <t xml:space="preserve"> 57101702301638396</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -892,15 +1042,21 @@
       <c r="C27" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D27" t="n">
-        <v>3135931234</v>
-      </c>
-      <c r="E27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696418</t>
+          <t xml:space="preserve"> 57101702301638395</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -909,15 +1065,21 @@
       <c r="C28" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D28" t="n">
-        <v>3135932083</v>
-      </c>
-      <c r="E28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696377</t>
+          <t xml:space="preserve"> 57101702301638394</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -926,15 +1088,21 @@
       <c r="C29" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D29" t="n">
-        <v>3135920930</v>
-      </c>
-      <c r="E29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696419</t>
+          <t xml:space="preserve"> 57101702301638393</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -943,15 +1111,21 @@
       <c r="C30" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D30" t="n">
-        <v>3135924354</v>
-      </c>
-      <c r="E30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696427</t>
+          <t xml:space="preserve"> 57101702301638392</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -960,15 +1134,21 @@
       <c r="C31" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D31" t="n">
-        <v>3135883979</v>
-      </c>
-      <c r="E31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696428</t>
+          <t xml:space="preserve"> 57101702301638391</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -977,15 +1157,21 @@
       <c r="C32" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D32" t="n">
-        <v>3135890241</v>
-      </c>
-      <c r="E32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696420</t>
+          <t xml:space="preserve"> 57101702301638390</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -994,15 +1180,21 @@
       <c r="C33" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D33" t="n">
-        <v>3135895342</v>
-      </c>
-      <c r="E33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696380</t>
+          <t xml:space="preserve"> 57101702301638389</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1011,15 +1203,21 @@
       <c r="C34" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D34" t="n">
-        <v>3135931271</v>
-      </c>
-      <c r="E34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696370</t>
+          <t xml:space="preserve"> 57101702301638388</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1028,15 +1226,21 @@
       <c r="C35" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D35" t="n">
-        <v>3135932600</v>
-      </c>
-      <c r="E35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696374</t>
+          <t xml:space="preserve"> 57101702301638387</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1045,15 +1249,21 @@
       <c r="C36" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D36" t="n">
-        <v>3135921779</v>
-      </c>
-      <c r="E36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696421</t>
+          <t xml:space="preserve"> 57101702301638386</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1062,15 +1272,21 @@
       <c r="C37" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D37" t="n">
-        <v>3135905263</v>
-      </c>
-      <c r="E37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696422</t>
+          <t xml:space="preserve"> 57101702301638464</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1079,15 +1295,21 @@
       <c r="C38" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D38" t="n">
-        <v>3135909078</v>
-      </c>
-      <c r="E38" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696372</t>
+          <t xml:space="preserve"> 57101702301638463</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1096,15 +1318,21 @@
       <c r="C39" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D39" t="n">
-        <v>3135915414</v>
-      </c>
-      <c r="E39" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696378</t>
+          <t xml:space="preserve"> 57101702301638462</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1113,15 +1341,21 @@
       <c r="C40" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D40" t="n">
-        <v>3135919178</v>
-      </c>
-      <c r="E40" t="inlineStr"/>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696425</t>
+          <t xml:space="preserve"> 57101702301638461</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1130,15 +1364,21 @@
       <c r="C41" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D41" t="n">
-        <v>3135884030</v>
-      </c>
-      <c r="E41" t="inlineStr"/>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696423</t>
+          <t xml:space="preserve"> 57101702301638460</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1147,15 +1387,21 @@
       <c r="C42" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D42" t="n">
-        <v>3135890364</v>
-      </c>
-      <c r="E42" t="inlineStr"/>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696371</t>
+          <t xml:space="preserve"> 57101702301638459</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1164,15 +1410,21 @@
       <c r="C43" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D43" t="n">
-        <v>3135896683</v>
-      </c>
-      <c r="E43" t="inlineStr"/>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696424</t>
+          <t xml:space="preserve"> 57101702301638458</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1181,15 +1433,21 @@
       <c r="C44" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D44" t="n">
-        <v>3135932194</v>
-      </c>
-      <c r="E44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696426</t>
+          <t xml:space="preserve"> 57101702301638457</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1198,15 +1456,17 @@
       <c r="C45" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D45" t="n">
-        <v>3135920374</v>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>3222868323</t>
+        </is>
       </c>
       <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696365</t>
+          <t xml:space="preserve"> 57101702301638456</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1215,15 +1475,21 @@
       <c r="C46" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D46" t="n">
-        <v>3135901604</v>
-      </c>
-      <c r="E46" t="inlineStr"/>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696363</t>
+          <t xml:space="preserve"> 57101602110142572</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1232,15 +1498,21 @@
       <c r="C47" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D47" t="n">
-        <v>3135911675</v>
-      </c>
-      <c r="E47" t="inlineStr"/>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696366</t>
+          <t xml:space="preserve"> 57101602110142573</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1249,15 +1521,21 @@
       <c r="C48" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D48" t="n">
-        <v>3135918062</v>
-      </c>
-      <c r="E48" t="inlineStr"/>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696367</t>
+          <t xml:space="preserve"> 57101602110142574</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1266,15 +1544,21 @@
       <c r="C49" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D49" t="n">
-        <v>3135881583</v>
-      </c>
-      <c r="E49" t="inlineStr"/>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101602706696368</t>
+          <t xml:space="preserve"> 57101502301625518</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1283,15 +1567,21 @@
       <c r="C50" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D50" t="n">
-        <v>3135891716</v>
-      </c>
-      <c r="E50" t="inlineStr"/>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638521</t>
+          <t xml:space="preserve"> 57101502301625487</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1300,15 +1590,21 @@
       <c r="C51" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D51" t="n">
-        <v>3135895450</v>
-      </c>
-      <c r="E51" t="inlineStr"/>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638520</t>
+          <t xml:space="preserve"> 57101502301625493</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1317,15 +1613,21 @@
       <c r="C52" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D52" t="n">
-        <v>3135932747</v>
-      </c>
-      <c r="E52" t="inlineStr"/>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638519</t>
+          <t xml:space="preserve"> 57101602002225877</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1334,15 +1636,21 @@
       <c r="C53" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D53" t="n">
-        <v>3135904168</v>
-      </c>
-      <c r="E53" t="inlineStr"/>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Validacion Causal Desactivacion IccId = Falso</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638518</t>
+          <t xml:space="preserve"> 57101602105408780</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1351,15 +1659,21 @@
       <c r="C54" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D54" t="n">
-        <v>3135909247</v>
-      </c>
-      <c r="E54" t="inlineStr"/>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638517</t>
+          <t xml:space="preserve"> 57101602002225886</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1368,15 +1682,21 @@
       <c r="C55" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D55" t="n">
-        <v>3135916835</v>
-      </c>
-      <c r="E55" t="inlineStr"/>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Validacion Causal Desactivacion IccId = Falso</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638542</t>
+          <t xml:space="preserve"> 57101602002225885</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1385,15 +1705,21 @@
       <c r="C56" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D56" t="n">
-        <v>3135880370</v>
-      </c>
-      <c r="E56" t="inlineStr"/>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Validacion Causal Desactivacion IccId = Falso</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638541</t>
+          <t xml:space="preserve"> 57101602002225884</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1402,15 +1728,21 @@
       <c r="C57" t="n">
         <v>1007477784</v>
       </c>
-      <c r="D57" t="n">
-        <v>3135891772</v>
-      </c>
-      <c r="E57" t="inlineStr"/>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Validacion Causal Desactivacion IccId = Falso</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638540</t>
+          <t xml:space="preserve"> 57101602002225991</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1421,15 +1753,19 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>3135918165</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Validacion Causal Desactivacion IccId = Falso</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638539</t>
+          <t xml:space="preserve"> 57101602110958883</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1440,15 +1776,19 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>3135881697</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638538</t>
+          <t xml:space="preserve"> 57101602110141974</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1459,15 +1799,19 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>3135893149</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638537</t>
+          <t xml:space="preserve"> 57101602008667085</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1478,15 +1822,19 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>3135932862</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Validacion Causal Desactivacion IccId = Falso</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638536</t>
+          <t xml:space="preserve"> 57101602110147232</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1497,15 +1845,19 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>3135903106</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638535</t>
+          <t xml:space="preserve"> 57101602109572025</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1516,15 +1868,19 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>3135915716</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638534</t>
+          <t xml:space="preserve"> 57101602109572022</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1535,15 +1891,19 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>3135919533</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638523</t>
+          <t xml:space="preserve"> 57101602109572023</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1554,15 +1914,19 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>3135927388</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638533</t>
+          <t xml:space="preserve"> 57101602109572021</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1573,15 +1937,19 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>3135883047</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638509</t>
+          <t xml:space="preserve"> 57101602109572020</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1592,15 +1960,19 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>3135889421</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638508</t>
+          <t xml:space="preserve"> 57101602106022369</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1611,15 +1983,19 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>3135893182</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638507</t>
+          <t xml:space="preserve"> 57101602110151617</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1630,15 +2006,19 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>3135898246</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Validacion Causal Desactivacion IccId = Falso</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638506</t>
+          <t xml:space="preserve"> 57101602110151700</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1649,15 +2029,19 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>3135922128</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638505</t>
+          <t xml:space="preserve"> 57101602110138436</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1668,15 +2052,19 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>3135901907</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638504</t>
+          <t xml:space="preserve"> 57101602110147018</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1687,15 +2075,19 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>3135909493</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638503</t>
+          <t xml:space="preserve"> 57101602110147099</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1706,15 +2098,19 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>3135915821</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638502</t>
+          <t xml:space="preserve"> 57101602109572488</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1725,15 +2121,19 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>3135923912</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638531</t>
+          <t xml:space="preserve"> 57101602110141980</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1744,15 +2144,19 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>3135880619</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638530</t>
+          <t xml:space="preserve"> 57101602110147226</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1763,15 +2167,19 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>3135884387</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638529</t>
+          <t xml:space="preserve"> 57101602110151618</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1782,15 +2190,19 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>3135893244</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638528</t>
+          <t xml:space="preserve"> 57101602110138433</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1801,15 +2213,19 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>3135922185</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638527</t>
+          <t xml:space="preserve"> 57101602105443071</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1820,15 +2236,19 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>3135909553</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638546</t>
+          <t xml:space="preserve"> 57101602106011823</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1839,15 +2259,19 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>3135915852</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638545</t>
+          <t xml:space="preserve"> 57101602106011819</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1858,15 +2282,19 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>3135923045</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638399</t>
+          <t xml:space="preserve"> 57101602106022702</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1877,15 +2305,19 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>3135927521</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638544</t>
+          <t xml:space="preserve"> 57101602106011824</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1896,15 +2328,19 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>3135880719</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638543</t>
+          <t xml:space="preserve"> 57101602110969362</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1920,14 +2356,14 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Validacion Causal Desactivacion IccId = Falso</t>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638571</t>
+          <t xml:space="preserve"> 57101602011955360</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1938,15 +2374,19 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>3135892118</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Validacion Causal Desactivacion IccId = Falso</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638570</t>
+          <t xml:space="preserve"> 57101602110969419</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1957,15 +2397,19 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>3135902069</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638569</t>
+          <t xml:space="preserve"> 57101602106022707</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1976,15 +2420,19 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>3135907128</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638568</t>
+          <t xml:space="preserve"> 57101602106022699</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1995,15 +2443,19 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>3135924895</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638567</t>
+          <t xml:space="preserve"> 57101602106022703</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -2014,15 +2466,19 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>3135927058</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638510</t>
+          <t xml:space="preserve"> 57101602105411446</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -2033,53 +2489,65 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>3135928582</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638562</t>
+          <t xml:space="preserve"> 57101602105442514</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>901306448</v>
+        <v>900721484</v>
       </c>
       <c r="C91" t="n">
         <v>1007477784</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>3135887126</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638561</t>
+          <t xml:space="preserve"> 57101602104733550</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>900721484</v>
+        <v>901306448</v>
       </c>
       <c r="C92" t="n">
         <v>1007477784</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>3135893416</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638560</t>
+          <t xml:space="preserve"> 57101602106011820</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -2090,15 +2558,19 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>3135900934</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638559</t>
+          <t xml:space="preserve"> 57101602106022698</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -2109,15 +2581,19 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>3135904651</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638558</t>
+          <t xml:space="preserve"> 57101602106011821</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -2128,15 +2604,19 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>3135910972</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638557</t>
+          <t xml:space="preserve"> 57101602106022700</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -2147,15 +2627,19 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>3135917285</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638556</t>
+          <t xml:space="preserve"> 57101602106022705</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -2166,15 +2650,19 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>3135924113</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638555</t>
+          <t xml:space="preserve"> 57101602110969415</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -2185,15 +2673,19 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>3135928620</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638554</t>
+          <t xml:space="preserve"> 57101602109591098</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2204,15 +2696,19 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>3135885949</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638553</t>
+          <t xml:space="preserve"> 57101602106011827</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2223,15 +2719,19 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>3135892252</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>ICC_ID - Identificación Tarjeta de Circuito Integrada.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702301638552</t>
+          <t xml:space="preserve"> 57101602012100081</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2242,105 +2742,14 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>3135898608</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr"/>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 57101702301638551</t>
-        </is>
-      </c>
-      <c r="B102" t="n">
-        <v>900721484</v>
-      </c>
-      <c r="C102" t="n">
-        <v>1007477784</v>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>3135903513</t>
-        </is>
-      </c>
-      <c r="E102" t="inlineStr"/>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 57101702301638550</t>
-        </is>
-      </c>
-      <c r="B103" t="n">
-        <v>901306448</v>
-      </c>
-      <c r="C103" t="n">
-        <v>1007477784</v>
-      </c>
-      <c r="D103" t="inlineStr">
-        <is>
-          <t>3135911047</t>
-        </is>
-      </c>
-      <c r="E103" t="inlineStr"/>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 57101702301638549</t>
-        </is>
-      </c>
-      <c r="B104" t="n">
-        <v>900721484</v>
-      </c>
-      <c r="C104" t="n">
-        <v>1007477784</v>
-      </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>3135918675</t>
-        </is>
-      </c>
-      <c r="E104" t="inlineStr"/>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 57101702301638548</t>
-        </is>
-      </c>
-      <c r="B105" t="n">
-        <v>901306448</v>
-      </c>
-      <c r="C105" t="n">
-        <v>1007477784</v>
-      </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>3135927741</t>
-        </is>
-      </c>
-      <c r="E105" t="inlineStr"/>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 57101702301638547</t>
-        </is>
-      </c>
-      <c r="B106" t="n">
-        <v>900721484</v>
-      </c>
-      <c r="C106" t="n">
-        <v>1007477784</v>
-      </c>
-      <c r="D106" t="inlineStr">
-        <is>
-          <t>3135929657</t>
-        </is>
-      </c>
-      <c r="E106" t="inlineStr"/>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Validacion Causal Desactivacion IccId = Falso</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Se solucionan novedades reportadas para el proceso de preactivador con respecto al login
</commit_message>
<xml_diff>
--- a/src/preactivador/preactivador.xlsx
+++ b/src/preactivador/preactivador.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E81"/>
+  <dimension ref="A1:E101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,7 +458,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037487</t>
+          <t xml:space="preserve"> 57101702403144727</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -468,14 +468,14 @@
         <v>1038626820</v>
       </c>
       <c r="D2" t="n">
-        <v>3204378369</v>
+        <v>3208842014</v>
       </c>
       <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037488</t>
+          <t xml:space="preserve"> 57101702403144728</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -485,14 +485,14 @@
         <v>1038626820</v>
       </c>
       <c r="D3" t="n">
-        <v>3204380859</v>
+        <v>3208810274</v>
       </c>
       <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037489</t>
+          <t xml:space="preserve"> 57101702403144729</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -502,14 +502,14 @@
         <v>1038626820</v>
       </c>
       <c r="D4" t="n">
-        <v>3204385879</v>
+        <v>3208780470</v>
       </c>
       <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037490</t>
+          <t xml:space="preserve"> 57101702403144730</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -518,17 +518,15 @@
       <c r="C5" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>3204388535</t>
-        </is>
+      <c r="D5" t="n">
+        <v>3208784299</v>
       </c>
       <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037491</t>
+          <t xml:space="preserve"> 57101702403144731</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -537,17 +535,15 @@
       <c r="C6" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>3204393550</t>
-        </is>
+      <c r="D6" t="n">
+        <v>3208812782</v>
       </c>
       <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037492</t>
+          <t xml:space="preserve"> 57101702403144732</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -556,17 +552,15 @@
       <c r="C7" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>3204394861</t>
-        </is>
+      <c r="D7" t="n">
+        <v>3208786367</v>
       </c>
       <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037493</t>
+          <t xml:space="preserve"> 57101702403144733</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -575,17 +569,15 @@
       <c r="C8" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>3204398670</t>
-        </is>
+      <c r="D8" t="n">
+        <v>3208787651</v>
       </c>
       <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037494</t>
+          <t xml:space="preserve"> 57101702403144734</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -594,17 +586,15 @@
       <c r="C9" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>3204325426</t>
-        </is>
+      <c r="D9" t="n">
+        <v>3208790150</v>
       </c>
       <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037497</t>
+          <t xml:space="preserve"> 57101702403144735</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -613,17 +603,15 @@
       <c r="C10" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>3204327968</t>
-        </is>
+      <c r="D10" t="n">
+        <v>3208792648</v>
       </c>
       <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037498</t>
+          <t xml:space="preserve"> 57101702403144736</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -632,17 +620,15 @@
       <c r="C11" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>3204331748</t>
-        </is>
+      <c r="D11" t="n">
+        <v>3208795168</v>
       </c>
       <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037499</t>
+          <t xml:space="preserve"> 57101702403144737</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -651,17 +637,15 @@
       <c r="C12" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>3204336809</t>
-        </is>
+      <c r="D12" t="n">
+        <v>3208798962</v>
       </c>
       <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037500</t>
+          <t xml:space="preserve"> 57101702403144738</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -670,17 +654,15 @@
       <c r="C13" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>3204341804</t>
-        </is>
+      <c r="D13" t="n">
+        <v>3208805363</v>
       </c>
       <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037501</t>
+          <t xml:space="preserve"> 57101702403144739</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -689,17 +671,15 @@
       <c r="C14" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>3204345611</t>
-        </is>
+      <c r="D14" t="n">
+        <v>3208809514</v>
       </c>
       <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037502</t>
+          <t xml:space="preserve"> 57101702403144740</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -708,17 +688,15 @@
       <c r="C15" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>3204350720</t>
-        </is>
+      <c r="D15" t="n">
+        <v>3208817807</v>
       </c>
       <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037503</t>
+          <t xml:space="preserve"> 57101702403144741</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -727,17 +705,15 @@
       <c r="C16" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>3204360763</t>
-        </is>
+      <c r="D16" t="n">
+        <v>3208778432</v>
       </c>
       <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037504</t>
+          <t xml:space="preserve"> 57101702403144742</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -746,17 +722,15 @@
       <c r="C17" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>3204367091</t>
-        </is>
+      <c r="D17" t="n">
+        <v>3208823103</v>
       </c>
       <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037505</t>
+          <t xml:space="preserve"> 57101702403144743</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -765,17 +739,15 @@
       <c r="C18" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>3204370908</t>
-        </is>
+      <c r="D18" t="n">
+        <v>3208829834</v>
       </c>
       <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037506</t>
+          <t xml:space="preserve"> 57101702403144744</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -784,17 +756,15 @@
       <c r="C19" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>3204375980</t>
-        </is>
+      <c r="D19" t="n">
+        <v>3208834174</v>
       </c>
       <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037507</t>
+          <t xml:space="preserve"> 57101702403144745</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -803,17 +773,15 @@
       <c r="C20" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>3204380995</t>
-        </is>
+      <c r="D20" t="n">
+        <v>3208836191</v>
       </c>
       <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037508</t>
+          <t xml:space="preserve"> 57101702403144746</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -822,17 +790,15 @@
       <c r="C21" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>3204384842</t>
-        </is>
+      <c r="D21" t="n">
+        <v>3208837108</v>
       </c>
       <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037509</t>
+          <t xml:space="preserve"> 57101702403144747</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -841,17 +807,15 @@
       <c r="C22" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>3204391136</t>
-        </is>
+      <c r="D22" t="n">
+        <v>3208838909</v>
       </c>
       <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037510</t>
+          <t xml:space="preserve"> 57101702403144748</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -860,17 +824,15 @@
       <c r="C23" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>3204394956</t>
-        </is>
+      <c r="D23" t="n">
+        <v>3208841389</v>
       </c>
       <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037511</t>
+          <t xml:space="preserve"> 57101702403144750</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -879,17 +841,15 @@
       <c r="C24" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>3204324240</t>
-        </is>
+      <c r="D24" t="n">
+        <v>3208845605</v>
       </c>
       <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037512</t>
+          <t xml:space="preserve"> 57101702403144751</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -898,17 +858,15 @@
       <c r="C25" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>3204331769</t>
-        </is>
+      <c r="D25" t="n">
+        <v>3208781785</v>
       </c>
       <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037513</t>
+          <t xml:space="preserve"> 57101702403144752</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -917,17 +875,15 @@
       <c r="C26" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>3204343160</t>
-        </is>
+      <c r="D26" t="n">
+        <v>3208786409</v>
       </c>
       <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037514</t>
+          <t xml:space="preserve"> 57101702403144753</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -936,17 +892,15 @@
       <c r="C27" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>3204353252</t>
-        </is>
+      <c r="D27" t="n">
+        <v>3208790237</v>
       </c>
       <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037515</t>
+          <t xml:space="preserve"> 57101702403144754</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -955,13 +909,15 @@
       <c r="C28" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D28" t="inlineStr"/>
+      <c r="D28" t="n">
+        <v>3208791473</v>
+      </c>
       <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037516</t>
+          <t xml:space="preserve"> 57101702403144755</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -970,13 +926,15 @@
       <c r="C29" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D29" t="inlineStr"/>
+      <c r="D29" t="n">
+        <v>3214796438</v>
+      </c>
       <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037517</t>
+          <t xml:space="preserve"> 57101702403144756</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -985,13 +943,15 @@
       <c r="C30" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D30" t="inlineStr"/>
+      <c r="D30" t="n">
+        <v>3214811698</v>
+      </c>
       <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037518</t>
+          <t xml:space="preserve"> 57101702403037470</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1000,13 +960,15 @@
       <c r="C31" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D31" t="inlineStr"/>
+      <c r="D31" t="n">
+        <v>3214750728</v>
+      </c>
       <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037519</t>
+          <t xml:space="preserve"> 57101702403037471</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1015,13 +977,15 @@
       <c r="C32" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D32" t="inlineStr"/>
+      <c r="D32" t="n">
+        <v>3214783861</v>
+      </c>
       <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037520</t>
+          <t xml:space="preserve"> 57101702403037472</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1030,13 +994,15 @@
       <c r="C33" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>3214800340</v>
+      </c>
       <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037531</t>
+          <t xml:space="preserve"> 57101702403037473</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1045,13 +1011,15 @@
       <c r="C34" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>3214802924</v>
+      </c>
       <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037532</t>
+          <t xml:space="preserve"> 57101702403037474</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1060,13 +1028,15 @@
       <c r="C35" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D35" t="inlineStr"/>
+      <c r="D35" t="n">
+        <v>3214763602</v>
+      </c>
       <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037521</t>
+          <t xml:space="preserve"> 57101702403037475</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1075,13 +1045,15 @@
       <c r="C36" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D36" t="inlineStr"/>
+      <c r="D36" t="n">
+        <v>3214785202</v>
+      </c>
       <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037522</t>
+          <t xml:space="preserve"> 57101702403037476</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1090,13 +1062,15 @@
       <c r="C37" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D37" t="inlineStr"/>
+      <c r="D37" t="n">
+        <v>3214786469</v>
+      </c>
       <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037528</t>
+          <t xml:space="preserve"> 57101702403037477</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1105,13 +1079,15 @@
       <c r="C38" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D38" t="inlineStr"/>
+      <c r="D38" t="n">
+        <v>3214787759</v>
+      </c>
       <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037529</t>
+          <t xml:space="preserve"> 57101702403037478</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1120,13 +1096,15 @@
       <c r="C39" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D39" t="inlineStr"/>
+      <c r="D39" t="n">
+        <v>3214791534</v>
+      </c>
       <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037530</t>
+          <t xml:space="preserve"> 57101702403037479</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1135,13 +1113,15 @@
       <c r="C40" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D40" t="inlineStr"/>
+      <c r="D40" t="n">
+        <v>3214808036</v>
+      </c>
       <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037533</t>
+          <t xml:space="preserve"> 57101702403037480</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1150,13 +1130,15 @@
       <c r="C41" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D41" t="inlineStr"/>
+      <c r="D41" t="n">
+        <v>3214740732</v>
+      </c>
       <c r="E41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037534</t>
+          <t xml:space="preserve"> 57101702403037481</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1165,13 +1147,15 @@
       <c r="C42" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D42" t="inlineStr"/>
+      <c r="D42" t="n">
+        <v>3214773904</v>
+      </c>
       <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037535</t>
+          <t xml:space="preserve"> 57101702403037482</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1180,13 +1164,15 @@
       <c r="C43" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D43" t="inlineStr"/>
+      <c r="D43" t="n">
+        <v>3214800515</v>
+      </c>
       <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037523</t>
+          <t xml:space="preserve"> 57101702403037483</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1195,13 +1181,15 @@
       <c r="C44" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D44" t="inlineStr"/>
+      <c r="D44" t="n">
+        <v>3214805638</v>
+      </c>
       <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037524</t>
+          <t xml:space="preserve"> 57101702403037484</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1210,13 +1198,15 @@
       <c r="C45" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D45" t="inlineStr"/>
+      <c r="D45" t="n">
+        <v>3214745893</v>
+      </c>
       <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037525</t>
+          <t xml:space="preserve"> 57101702403037485</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1225,13 +1215,15 @@
       <c r="C46" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D46" t="inlineStr"/>
+      <c r="D46" t="n">
+        <v>3214795541</v>
+      </c>
       <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037526</t>
+          <t xml:space="preserve"> 57101702403037486</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1240,13 +1232,15 @@
       <c r="C47" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D47" t="inlineStr"/>
+      <c r="D47" t="n">
+        <v>3214809464</v>
+      </c>
       <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037527</t>
+          <t xml:space="preserve"> 57101702403037515</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1255,13 +1249,15 @@
       <c r="C48" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D48" t="inlineStr"/>
+      <c r="D48" t="n">
+        <v>3214809487</v>
+      </c>
       <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037536</t>
+          <t xml:space="preserve"> 57101702403037516</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1270,13 +1266,15 @@
       <c r="C49" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>3214810792</v>
+      </c>
       <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037537</t>
+          <t xml:space="preserve"> 57101702403037517</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1285,13 +1283,15 @@
       <c r="C50" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D50" t="inlineStr"/>
+      <c r="D50" t="n">
+        <v>3214744681</v>
+      </c>
       <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037538</t>
+          <t xml:space="preserve"> 57101702403037518</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1300,13 +1300,15 @@
       <c r="C51" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D51" t="inlineStr"/>
+      <c r="D51" t="n">
+        <v>3214771569</v>
+      </c>
       <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037539</t>
+          <t xml:space="preserve"> 57101702403037519</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1315,13 +1317,15 @@
       <c r="C52" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D52" t="inlineStr"/>
+      <c r="D52" t="n">
+        <v>3214785487</v>
+      </c>
       <c r="E52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037540</t>
+          <t xml:space="preserve"> 57101702403037520</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1330,13 +1334,15 @@
       <c r="C53" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D53" t="inlineStr"/>
+      <c r="D53" t="n">
+        <v>3214823435</v>
+      </c>
       <c r="E53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037541</t>
+          <t xml:space="preserve"> 57101702403037531</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1345,13 +1351,15 @@
       <c r="C54" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D54" t="inlineStr"/>
+      <c r="D54" t="n">
+        <v>3214841137</v>
+      </c>
       <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037542</t>
+          <t xml:space="preserve"> 57101702403037532</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1360,13 +1368,15 @@
       <c r="C55" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D55" t="inlineStr"/>
+      <c r="D55" t="n">
+        <v>3214856360</v>
+      </c>
       <c r="E55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037543</t>
+          <t xml:space="preserve"> 57101702403037521</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1375,13 +1385,15 @@
       <c r="C56" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D56" t="inlineStr"/>
+      <c r="D56" t="n">
+        <v>3214860121</v>
+      </c>
       <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037544</t>
+          <t xml:space="preserve"> 57101702403037522</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1390,13 +1402,17 @@
       <c r="C57" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D57" t="inlineStr"/>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>3214849118</t>
+        </is>
+      </c>
       <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037545</t>
+          <t xml:space="preserve"> 57101702403037528</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1405,13 +1421,17 @@
       <c r="C58" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D58" t="inlineStr"/>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>3214890977</t>
+        </is>
+      </c>
       <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037546</t>
+          <t xml:space="preserve"> 57101702403037529</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1420,13 +1440,17 @@
       <c r="C59" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D59" t="inlineStr"/>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>3214835320</t>
+        </is>
+      </c>
       <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037547</t>
+          <t xml:space="preserve"> 57101702403037530</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1435,13 +1459,17 @@
       <c r="C60" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D60" t="inlineStr"/>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>3214840349</t>
+        </is>
+      </c>
       <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037548</t>
+          <t xml:space="preserve"> 57101702403037533</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1450,13 +1478,17 @@
       <c r="C61" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D61" t="inlineStr"/>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>3214853053</t>
+        </is>
+      </c>
       <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037549</t>
+          <t xml:space="preserve"> 57101702403037534</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1465,13 +1497,17 @@
       <c r="C62" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D62" t="inlineStr"/>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>3214874545</t>
+        </is>
+      </c>
       <c r="E62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037550</t>
+          <t xml:space="preserve"> 57101702403037535</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1480,13 +1516,17 @@
       <c r="C63" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D63" t="inlineStr"/>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>3214882151</t>
+        </is>
+      </c>
       <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037551</t>
+          <t xml:space="preserve"> 57101702403037523</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1495,13 +1535,17 @@
       <c r="C64" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D64" t="inlineStr"/>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>3214885941</t>
+        </is>
+      </c>
       <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037553</t>
+          <t xml:space="preserve"> 57101702403037524</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1510,13 +1554,17 @@
       <c r="C65" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D65" t="inlineStr"/>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>3214885986</t>
+        </is>
+      </c>
       <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037554</t>
+          <t xml:space="preserve"> 57101702403037525</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1531,7 +1579,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037555</t>
+          <t xml:space="preserve"> 57101702403037526</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1540,13 +1588,17 @@
       <c r="C67" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D67" t="inlineStr"/>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>3214892258</t>
+        </is>
+      </c>
       <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037556</t>
+          <t xml:space="preserve"> 57101702403037527</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1555,13 +1607,17 @@
       <c r="C68" t="n">
         <v>1038626820</v>
       </c>
-      <c r="D68" t="inlineStr"/>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>3214894815</t>
+        </is>
+      </c>
       <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037557</t>
+          <t xml:space="preserve"> 57101702403037536</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1576,7 +1632,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037558</t>
+          <t xml:space="preserve"> 57101702403037537</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1591,7 +1647,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037559</t>
+          <t xml:space="preserve"> 57101702403037538</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1606,7 +1662,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037560</t>
+          <t xml:space="preserve"> 57101702403037539</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1621,7 +1677,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037561</t>
+          <t xml:space="preserve"> 57101702403037540</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1636,7 +1692,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037562</t>
+          <t xml:space="preserve"> 57101702403037541</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1651,7 +1707,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037563</t>
+          <t xml:space="preserve"> 57101702403037542</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1666,7 +1722,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037564</t>
+          <t xml:space="preserve"> 57101702403037543</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1681,7 +1737,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037565</t>
+          <t xml:space="preserve"> 57101702403037544</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1696,7 +1752,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037566</t>
+          <t xml:space="preserve"> 57101702403037545</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1711,7 +1767,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037567</t>
+          <t xml:space="preserve"> 57101702403037546</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1726,7 +1782,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037468</t>
+          <t xml:space="preserve"> 57101702403037547</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1741,7 +1797,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702403037469</t>
+          <t xml:space="preserve"> 57101702403037548</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1752,6 +1808,306 @@
       </c>
       <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702403037549</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>901306448</v>
+      </c>
+      <c r="C82" t="n">
+        <v>1038626820</v>
+      </c>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702403037550</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>900721484</v>
+      </c>
+      <c r="C83" t="n">
+        <v>1038626820</v>
+      </c>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702403037551</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>901306448</v>
+      </c>
+      <c r="C84" t="n">
+        <v>1038626820</v>
+      </c>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702403037553</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>900721484</v>
+      </c>
+      <c r="C85" t="n">
+        <v>1038626820</v>
+      </c>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702403037554</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>901306448</v>
+      </c>
+      <c r="C86" t="n">
+        <v>1038626820</v>
+      </c>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702403037555</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>900721484</v>
+      </c>
+      <c r="C87" t="n">
+        <v>1038626820</v>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702403037556</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>901306448</v>
+      </c>
+      <c r="C88" t="n">
+        <v>1038626820</v>
+      </c>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702403037557</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>900721484</v>
+      </c>
+      <c r="C89" t="n">
+        <v>1038626820</v>
+      </c>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702403037558</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>901306448</v>
+      </c>
+      <c r="C90" t="n">
+        <v>1038626820</v>
+      </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702403037559</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>900721484</v>
+      </c>
+      <c r="C91" t="n">
+        <v>1038626820</v>
+      </c>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702403037560</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>901306448</v>
+      </c>
+      <c r="C92" t="n">
+        <v>1038626820</v>
+      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702403037561</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>900721484</v>
+      </c>
+      <c r="C93" t="n">
+        <v>1038626820</v>
+      </c>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702403037562</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>901306448</v>
+      </c>
+      <c r="C94" t="n">
+        <v>1038626820</v>
+      </c>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702403037563</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>900721484</v>
+      </c>
+      <c r="C95" t="n">
+        <v>1038626820</v>
+      </c>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702403037564</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>901306448</v>
+      </c>
+      <c r="C96" t="n">
+        <v>1038626820</v>
+      </c>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702403037565</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>900721484</v>
+      </c>
+      <c r="C97" t="n">
+        <v>1038626820</v>
+      </c>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702403037566</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>901306448</v>
+      </c>
+      <c r="C98" t="n">
+        <v>1038626820</v>
+      </c>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702403037567</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>900721484</v>
+      </c>
+      <c r="C99" t="n">
+        <v>1038626820</v>
+      </c>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702403037468</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>901306448</v>
+      </c>
+      <c r="C100" t="n">
+        <v>1038626820</v>
+      </c>
+      <c r="D100" t="inlineStr"/>
+      <c r="E100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702403037469</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>900721484</v>
+      </c>
+      <c r="C101" t="n">
+        <v>1038626820</v>
+      </c>
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Implementación de panel de control para tiempo de espera entre transacciones
</commit_message>
<xml_diff>
--- a/src/preactivador/preactivador.xlsx
+++ b/src/preactivador/preactivador.xlsx
@@ -609,7 +609,11 @@
       <c r="D8" t="n">
         <v>1038626820</v>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>3108529292</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
@@ -959,10 +963,8 @@
       <c r="D24" t="n">
         <v>1038626820</v>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>3102863516</t>
-        </is>
+      <c r="E24" t="n">
+        <v>3102863516</v>
       </c>
       <c r="F24" t="inlineStr"/>
     </row>

</xml_diff>